<commit_message>
feat(blog): drei Beitraege als Entwuerfe — bewusst NICHT eingehaengt (keine Sidebar/Teaser/Sitemap/Feeds/Twins)
- 2026/08/21 testing-a-saas-with-nanook (Feldbericht; Marker-Semantik nach Nanook-Doku,
  Generator- und Flow-Abschnitt, dasHandwerk verlinkt)
- 2026/08/22 login-example-ai-generated-table (Worked Example; Tabelle/Daten aus echtem Lauf,
  prds/assets/login-example regeneriert mit CASCADE-Markern)
- 2026/08/29 e-invoicing-decision-tables
- 7 SVG-Diagramme unter img/blog/ (dunkles Theme, CSS-Invert)
- PRD-Nachtraege (Marker-Korrektur 08-30, dasHandwerk-Link 08-31) + zwei LinkedIn-Paste-Texte

Erreichbar nur per Direkt-URL; Registrierung an den sechs Stellen folgt nach Freigabe.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011j6M6J1bpGXepDKM93gi4u
</commit_message>
<xml_diff>
--- a/prds/assets/login-example/login.xlsx
+++ b/prds/assets/login-example/login.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M25"/>
+  <dimension ref="A1:M26"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -838,16 +838,16 @@
         <v/>
       </c>
       <c r="J11" t="str">
+        <v>x</v>
+      </c>
+      <c r="K11" t="str">
+        <v>x</v>
+      </c>
+      <c r="L11" t="str">
         <v>a</v>
       </c>
-      <c r="K11" t="str">
+      <c r="M11" t="str">
         <v>a</v>
-      </c>
-      <c r="L11" t="str">
-        <v>x</v>
-      </c>
-      <c r="M11" t="str">
-        <v>x</v>
       </c>
     </row>
     <row r="12">
@@ -885,10 +885,10 @@
         <v/>
       </c>
       <c r="L12" t="str">
-        <v/>
+        <v>e</v>
       </c>
       <c r="M12" t="str">
-        <v/>
+        <v>e</v>
       </c>
     </row>
     <row r="13">
@@ -926,10 +926,10 @@
         <v/>
       </c>
       <c r="L13" t="str">
-        <v/>
+        <v>e</v>
       </c>
       <c r="M13" t="str">
-        <v/>
+        <v>e</v>
       </c>
     </row>
     <row r="14">
@@ -967,10 +967,10 @@
         <v/>
       </c>
       <c r="L14" t="str">
-        <v/>
+        <v>e</v>
       </c>
       <c r="M14" t="str">
-        <v/>
+        <v>e</v>
       </c>
     </row>
     <row r="15">
@@ -1049,10 +1049,10 @@
         <v/>
       </c>
       <c r="L16" t="str">
-        <v>x</v>
+        <v>a</v>
       </c>
       <c r="M16" t="str">
-        <v>x</v>
+        <v>a</v>
       </c>
     </row>
     <row r="17">
@@ -1075,13 +1075,13 @@
         <v/>
       </c>
       <c r="G17" t="str">
-        <v/>
+        <v>e</v>
       </c>
       <c r="H17" t="str">
-        <v/>
+        <v>e</v>
       </c>
       <c r="I17" t="str">
-        <v/>
+        <v>e</v>
       </c>
       <c r="J17" t="str">
         <v>x</v>
@@ -1090,10 +1090,10 @@
         <v/>
       </c>
       <c r="L17" t="str">
-        <v/>
+        <v>e</v>
       </c>
       <c r="M17" t="str">
-        <v/>
+        <v>e</v>
       </c>
     </row>
     <row r="18">
@@ -1116,13 +1116,13 @@
         <v/>
       </c>
       <c r="G18" t="str">
-        <v/>
+        <v>e</v>
       </c>
       <c r="H18" t="str">
-        <v/>
+        <v>e</v>
       </c>
       <c r="I18" t="str">
-        <v/>
+        <v>e</v>
       </c>
       <c r="J18" t="str">
         <v/>
@@ -1131,10 +1131,10 @@
         <v>x</v>
       </c>
       <c r="L18" t="str">
-        <v/>
+        <v>e</v>
       </c>
       <c r="M18" t="str">
-        <v/>
+        <v>e</v>
       </c>
     </row>
     <row r="19">
@@ -1356,10 +1356,10 @@
         <v/>
       </c>
       <c r="E24" t="str">
-        <v>SOLL: only for a real account with a wrong password — not for an unknown one</v>
+        <v>real account, wrong password</v>
       </c>
       <c r="F24" t="str">
-        <v>e</v>
+        <v/>
       </c>
       <c r="G24" t="str">
         <v/>
@@ -1377,7 +1377,7 @@
         <v>x</v>
       </c>
       <c r="L24" t="str">
-        <v>e</v>
+        <v/>
       </c>
       <c r="M24" t="str">
         <v/>
@@ -1385,48 +1385,89 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
+        <v/>
+      </c>
+      <c r="B25" t="str">
+        <v/>
+      </c>
+      <c r="C25" t="str">
+        <v>failed-attempt counter unchanged</v>
+      </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
+      <c r="E25" t="str">
+        <v>success or unknown user</v>
+      </c>
+      <c r="F25" t="str">
+        <v>x</v>
+      </c>
+      <c r="G25" t="str">
+        <v/>
+      </c>
+      <c r="H25" t="str">
+        <v/>
+      </c>
+      <c r="I25" t="str">
+        <v/>
+      </c>
+      <c r="J25" t="str">
+        <v/>
+      </c>
+      <c r="K25" t="str">
+        <v/>
+      </c>
+      <c r="L25" t="str">
+        <v>x</v>
+      </c>
+      <c r="M25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
         <v>&lt;END&gt;</v>
       </c>
-      <c r="B25" t="str">
-        <v/>
-      </c>
-      <c r="C25" t="str">
-        <v/>
-      </c>
-      <c r="D25" t="str">
-        <v/>
-      </c>
-      <c r="E25" t="str">
-        <v/>
-      </c>
-      <c r="F25" t="str">
-        <v/>
-      </c>
-      <c r="G25" t="str">
-        <v/>
-      </c>
-      <c r="H25" t="str">
-        <v/>
-      </c>
-      <c r="I25" t="str">
-        <v/>
-      </c>
-      <c r="J25" t="str">
-        <v/>
-      </c>
-      <c r="K25" t="str">
-        <v/>
-      </c>
-      <c r="L25" t="str">
-        <v/>
-      </c>
-      <c r="M25" t="str">
+      <c r="B26" t="str">
+        <v/>
+      </c>
+      <c r="C26" t="str">
+        <v/>
+      </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
+      <c r="F26" t="str">
+        <v/>
+      </c>
+      <c r="G26" t="str">
+        <v/>
+      </c>
+      <c r="H26" t="str">
+        <v/>
+      </c>
+      <c r="I26" t="str">
+        <v/>
+      </c>
+      <c r="J26" t="str">
+        <v/>
+      </c>
+      <c r="K26" t="str">
+        <v/>
+      </c>
+      <c r="L26" t="str">
+        <v/>
+      </c>
+      <c r="M26" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M26"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>